<commit_message>
Release v1.0.29: improve reading, raids and collection overlay
</commit_message>
<xml_diff>
--- a/docs/revisao-iv-master-nivel-40.xlsx
+++ b/docs/revisao-iv-master-nivel-40.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12300" activeTab="3"/>
+    <workbookView windowWidth="28800" windowHeight="12300" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Orientações" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1641" uniqueCount="544">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1639" uniqueCount="544">
   <si>
     <t>PLANILHA DE REVISÃO IV MASTER</t>
   </si>
@@ -587,217 +587,217 @@
     <t>Proposta para o alvo indicado, por produto de atributos no nível 40; confirmar evolução/forma.</t>
   </si>
   <si>
+    <t>F-002</t>
+  </si>
+  <si>
+    <t>Raichu (Alola)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=RAICHU_ALOLA</t>
+  </si>
+  <si>
+    <t>F-003</t>
+  </si>
+  <si>
+    <t>Sandshrew (Alola) / Sandslash (Alola)</t>
+  </si>
+  <si>
+    <t>Sandshrew (Alola); Sandslash (Alola)</t>
+  </si>
+  <si>
+    <t>Sandslash (Alola)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=SANDSLASH_ALOLA</t>
+  </si>
+  <si>
+    <t>F-004</t>
+  </si>
+  <si>
+    <t>Vulpix (Alola) / Ninetales (Alola)</t>
+  </si>
+  <si>
+    <t>Vulpix (Alola); Ninetales (Alola)</t>
+  </si>
+  <si>
+    <t>Ninetales (Alola)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=NINETALES_ALOLA</t>
+  </si>
+  <si>
+    <t>F-005</t>
+  </si>
+  <si>
+    <t>Diglett (Alola) / Dugtrio (Alola)</t>
+  </si>
+  <si>
+    <t>Diglett (Alola); Dugtrio (Alola)</t>
+  </si>
+  <si>
+    <t>Dugtrio (Alola)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=DUGTRIO_ALOLA</t>
+  </si>
+  <si>
+    <t>F-006</t>
+  </si>
+  <si>
+    <t>Meowth (Alola) / Persian (Alola)</t>
+  </si>
+  <si>
+    <t>Meowth (Alola); Persian (Alola)</t>
+  </si>
+  <si>
+    <t>Persian (Alola)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=PERSIAN_ALOLA</t>
+  </si>
+  <si>
+    <t>F-007</t>
+  </si>
+  <si>
+    <t>Growlithe (Hisui) / Arcanine (Hisui)</t>
+  </si>
+  <si>
+    <t>Growlithe (Hisui); Arcanine (Hisui)</t>
+  </si>
+  <si>
+    <t>Arcanine (Hisui)</t>
+  </si>
+  <si>
+    <t>14/15/12</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=ARCANINE_HISUIAN</t>
+  </si>
+  <si>
+    <t>F-008</t>
+  </si>
+  <si>
+    <t>Geodude (Alola) / Graveler (Alola) / Golem (Alola)</t>
+  </si>
+  <si>
+    <t>Geodude (Alola); Graveler (Alola); Golem (Alola)</t>
+  </si>
+  <si>
+    <t>Golem (Alola)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=GOLEM_ALOLA</t>
+  </si>
+  <si>
+    <t>F-009</t>
+  </si>
+  <si>
+    <t>Ponyta (Galar) / Rapidash (Galar)</t>
+  </si>
+  <si>
+    <t>Ponyta (Galar); Rapidash (Galar)</t>
+  </si>
+  <si>
+    <t>Rapidash (Galar)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=RAPIDASH_GALARIAN</t>
+  </si>
+  <si>
+    <t>F-010</t>
+  </si>
+  <si>
+    <t>Slowpoke (Galar) / Slowbro (Galar) / Slowking (Galar)</t>
+  </si>
+  <si>
+    <t>Slowpoke (Galar); Slowbro (Galar); Slowking (Galar)</t>
+  </si>
+  <si>
+    <t>Slowking (Galar)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=SLOWKING_GALARIAN</t>
+  </si>
+  <si>
+    <t>F-011</t>
+  </si>
+  <si>
+    <t>Grimer (Alola) / Muk (Alola)</t>
+  </si>
+  <si>
+    <t>Grimer (Alola); Muk (Alola)</t>
+  </si>
+  <si>
+    <t>Muk (Alola)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=MUK_ALOLA</t>
+  </si>
+  <si>
+    <t>F-012</t>
+  </si>
+  <si>
+    <t>Voltorb (Hisui) / Electrode (Hisui)</t>
+  </si>
+  <si>
+    <t>Voltorb (Hisui); Electrode (Hisui)</t>
+  </si>
+  <si>
+    <t>Electrode (Hisui)</t>
+  </si>
+  <si>
+    <t>14/15/15 ou 15/14/15</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=ELECTRODE_HISUIAN</t>
+  </si>
+  <si>
+    <t>F-013</t>
+  </si>
+  <si>
+    <t>Exeggutor (Alola)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=EXEGGUTOR_ALOLA</t>
+  </si>
+  <si>
+    <t>F-014</t>
+  </si>
+  <si>
+    <t>Marowak (Alola)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=MAROWAK_ALOLA</t>
+  </si>
+  <si>
+    <t>F-015</t>
+  </si>
+  <si>
+    <t>Weezing (Galar)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=WEEZING_GALARIAN</t>
+  </si>
+  <si>
+    <t>F-016</t>
+  </si>
+  <si>
+    <t>Tauros (Paldea)</t>
+  </si>
+  <si>
+    <t>Sem atributos/correspondência inequívoca no Stadium; validar manualmente.</t>
+  </si>
+  <si>
+    <t>F-017</t>
+  </si>
+  <si>
+    <t>Articuno (Galar)</t>
+  </si>
+  <si>
+    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=ARTICUNO_GALARIAN</t>
+  </si>
+  <si>
     <t>Pendente</t>
-  </si>
-  <si>
-    <t>F-002</t>
-  </si>
-  <si>
-    <t>Raichu (Alola)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=RAICHU_ALOLA</t>
-  </si>
-  <si>
-    <t>F-003</t>
-  </si>
-  <si>
-    <t>Sandshrew (Alola) / Sandslash (Alola)</t>
-  </si>
-  <si>
-    <t>Sandshrew (Alola); Sandslash (Alola)</t>
-  </si>
-  <si>
-    <t>Sandslash (Alola)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=SANDSLASH_ALOLA</t>
-  </si>
-  <si>
-    <t>F-004</t>
-  </si>
-  <si>
-    <t>Vulpix (Alola) / Ninetales (Alola)</t>
-  </si>
-  <si>
-    <t>Vulpix (Alola); Ninetales (Alola)</t>
-  </si>
-  <si>
-    <t>Ninetales (Alola)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=NINETALES_ALOLA</t>
-  </si>
-  <si>
-    <t>F-005</t>
-  </si>
-  <si>
-    <t>Diglett (Alola) / Dugtrio (Alola)</t>
-  </si>
-  <si>
-    <t>Diglett (Alola); Dugtrio (Alola)</t>
-  </si>
-  <si>
-    <t>Dugtrio (Alola)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=DUGTRIO_ALOLA</t>
-  </si>
-  <si>
-    <t>F-006</t>
-  </si>
-  <si>
-    <t>Meowth (Alola) / Persian (Alola)</t>
-  </si>
-  <si>
-    <t>Meowth (Alola); Persian (Alola)</t>
-  </si>
-  <si>
-    <t>Persian (Alola)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=PERSIAN_ALOLA</t>
-  </si>
-  <si>
-    <t>F-007</t>
-  </si>
-  <si>
-    <t>Growlithe (Hisui) / Arcanine (Hisui)</t>
-  </si>
-  <si>
-    <t>Growlithe (Hisui); Arcanine (Hisui)</t>
-  </si>
-  <si>
-    <t>Arcanine (Hisui)</t>
-  </si>
-  <si>
-    <t>14/15/12</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=ARCANINE_HISUIAN</t>
-  </si>
-  <si>
-    <t>F-008</t>
-  </si>
-  <si>
-    <t>Geodude (Alola) / Graveler (Alola) / Golem (Alola)</t>
-  </si>
-  <si>
-    <t>Geodude (Alola); Graveler (Alola); Golem (Alola)</t>
-  </si>
-  <si>
-    <t>Golem (Alola)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=GOLEM_ALOLA</t>
-  </si>
-  <si>
-    <t>F-009</t>
-  </si>
-  <si>
-    <t>Ponyta (Galar) / Rapidash (Galar)</t>
-  </si>
-  <si>
-    <t>Ponyta (Galar); Rapidash (Galar)</t>
-  </si>
-  <si>
-    <t>Rapidash (Galar)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=RAPIDASH_GALARIAN</t>
-  </si>
-  <si>
-    <t>F-010</t>
-  </si>
-  <si>
-    <t>Slowpoke (Galar) / Slowbro (Galar) / Slowking (Galar)</t>
-  </si>
-  <si>
-    <t>Slowpoke (Galar); Slowbro (Galar); Slowking (Galar)</t>
-  </si>
-  <si>
-    <t>Slowking (Galar)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=SLOWKING_GALARIAN</t>
-  </si>
-  <si>
-    <t>F-011</t>
-  </si>
-  <si>
-    <t>Grimer (Alola) / Muk (Alola)</t>
-  </si>
-  <si>
-    <t>Grimer (Alola); Muk (Alola)</t>
-  </si>
-  <si>
-    <t>Muk (Alola)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=MUK_ALOLA</t>
-  </si>
-  <si>
-    <t>F-012</t>
-  </si>
-  <si>
-    <t>Voltorb (Hisui) / Electrode (Hisui)</t>
-  </si>
-  <si>
-    <t>Voltorb (Hisui); Electrode (Hisui)</t>
-  </si>
-  <si>
-    <t>Electrode (Hisui)</t>
-  </si>
-  <si>
-    <t>14/15/15 ou 15/14/15</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=ELECTRODE_HISUIAN</t>
-  </si>
-  <si>
-    <t>F-013</t>
-  </si>
-  <si>
-    <t>Exeggutor (Alola)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=EXEGGUTOR_ALOLA</t>
-  </si>
-  <si>
-    <t>F-014</t>
-  </si>
-  <si>
-    <t>Marowak (Alola)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=MAROWAK_ALOLA</t>
-  </si>
-  <si>
-    <t>F-015</t>
-  </si>
-  <si>
-    <t>Weezing (Galar)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=WEEZING_GALARIAN</t>
-  </si>
-  <si>
-    <t>F-016</t>
-  </si>
-  <si>
-    <t>Tauros (Paldea)</t>
-  </si>
-  <si>
-    <t>Sem atributos/correspondência inequívoca no Stadium; validar manualmente.</t>
-  </si>
-  <si>
-    <t>F-017</t>
-  </si>
-  <si>
-    <t>Articuno (Galar)</t>
-  </si>
-  <si>
-    <t>https://www.stadiumgaming.gg/rank-checker?pokemon=ARTICUNO_GALARIAN</t>
   </si>
   <si>
     <t>F-018</t>
@@ -2316,7 +2316,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2331,6 +2331,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2923,9 +2926,11 @@
   <dimension ref="A1:K33"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="6" width="18" customWidth="1"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="16.2857142857143" customWidth="1"/>
+    <col min="3" max="4" width="13.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="12.2857142857143" customWidth="1"/>
+    <col min="6" max="6" width="13.4285714285714" customWidth="1"/>
     <col min="7" max="7" width="55" customWidth="1"/>
     <col min="8" max="8" width="25" customWidth="1"/>
     <col min="9" max="10" width="18" customWidth="1"/>
@@ -3486,7 +3491,7 @@
         <v>44</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>45</v>
@@ -3521,7 +3526,7 @@
         <v>44</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="K17" s="3" t="s">
         <v>45</v>
@@ -3556,7 +3561,7 @@
         <v>44</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="K18" s="3" t="s">
         <v>45</v>
@@ -3591,7 +3596,7 @@
         <v>44</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="K19" s="3" t="s">
         <v>45</v>
@@ -3626,7 +3631,7 @@
         <v>44</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="K20" s="3" t="s">
         <v>45</v>
@@ -3661,7 +3666,7 @@
         <v>44</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>45</v>
+        <v>110</v>
       </c>
       <c r="K21" s="3" t="s">
         <v>45</v>
@@ -3696,7 +3701,7 @@
         <v>44</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>45</v>
+        <v>114</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>45</v>
@@ -3731,7 +3736,7 @@
         <v>44</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>45</v>
+        <v>117</v>
       </c>
       <c r="K23" s="3" t="s">
         <v>45</v>
@@ -3766,7 +3771,7 @@
         <v>44</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="K24" s="3" t="s">
         <v>45</v>
@@ -3801,7 +3806,7 @@
         <v>44</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="K25" s="3" t="s">
         <v>45</v>
@@ -3836,7 +3841,7 @@
         <v>44</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>45</v>
+        <v>56</v>
       </c>
       <c r="K26" s="3" t="s">
         <v>45</v>
@@ -3871,7 +3876,7 @@
         <v>44</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="K27" s="3" t="s">
         <v>45</v>
@@ -3905,8 +3910,8 @@
       <c r="I28" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J28" s="3" t="s">
-        <v>45</v>
+      <c r="J28" s="6">
+        <v>42353</v>
       </c>
       <c r="K28" s="3" t="s">
         <v>45</v>
@@ -3941,7 +3946,7 @@
         <v>44</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="K29" s="3" t="s">
         <v>45</v>
@@ -3976,7 +3981,7 @@
         <v>44</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="K30" s="3" t="s">
         <v>45</v>
@@ -4089,7 +4094,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="I6 I2:I5 I7:I33">
+    <dataValidation type="list" sqref="I2:I33">
       <formula1>"Pendente,Aprovar proposta,Manter atual,Definir outro IV,Revisar forma/família"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4459,10 +4464,15 @@
   <dimension ref="A1:Q47"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="3" width="55" customWidth="1"/>
-    <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="9" width="18" customWidth="1"/>
+    <col min="1" max="1" width="7.14285714285714" customWidth="1"/>
+    <col min="2" max="2" width="29" customWidth="1"/>
+    <col min="3" max="3" width="28.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="16.8571428571429" customWidth="1"/>
+    <col min="5" max="5" width="15.1428571428571" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="12.4285714285714" customWidth="1"/>
+    <col min="8" max="8" width="12.2857142857143" customWidth="1"/>
+    <col min="9" max="9" width="12.1428571428571" customWidth="1"/>
     <col min="10" max="10" width="25" customWidth="1"/>
     <col min="11" max="11" width="55" customWidth="1"/>
     <col min="12" max="16" width="18" customWidth="1"/>
@@ -4557,7 +4567,7 @@
         <v>183</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>45</v>
@@ -4577,16 +4587,16 @@
     </row>
     <row r="3" ht="62" customHeight="1" spans="1:17">
       <c r="A3" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>186</v>
-      </c>
       <c r="C3" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>179</v>
@@ -4604,13 +4614,13 @@
         <v>95</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>45</v>
@@ -4630,16 +4640,16 @@
     </row>
     <row r="4" ht="62" customHeight="1" spans="1:17">
       <c r="A4" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>190</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>191</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>179</v>
@@ -4657,13 +4667,13 @@
         <v>181</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>45</v>
@@ -4683,16 +4693,16 @@
     </row>
     <row r="5" ht="62" customHeight="1" spans="1:17">
       <c r="A5" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>196</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>179</v>
@@ -4710,13 +4720,13 @@
         <v>72</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M5" s="3" t="s">
         <v>45</v>
@@ -4736,16 +4746,16 @@
     </row>
     <row r="6" ht="62" customHeight="1" spans="1:17">
       <c r="A6" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>201</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>179</v>
@@ -4763,13 +4773,13 @@
         <v>95</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>45</v>
@@ -4789,16 +4799,16 @@
     </row>
     <row r="7" ht="62" customHeight="1" spans="1:17">
       <c r="A7" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>206</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>179</v>
@@ -4816,13 +4826,13 @@
         <v>56</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M7" s="3" t="s">
         <v>45</v>
@@ -4842,16 +4852,16 @@
     </row>
     <row r="8" ht="62" customHeight="1" spans="1:17">
       <c r="A8" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>208</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>211</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>179</v>
@@ -4866,16 +4876,16 @@
         <v>64</v>
       </c>
       <c r="I8" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="J8" s="4" t="s">
         <v>212</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>213</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M8" s="3" t="s">
         <v>45</v>
@@ -4895,16 +4905,16 @@
     </row>
     <row r="9" ht="62" customHeight="1" spans="1:17">
       <c r="A9" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>216</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>217</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>179</v>
@@ -4922,13 +4932,13 @@
         <v>95</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>45</v>
@@ -4948,16 +4958,16 @@
     </row>
     <row r="10" ht="62" customHeight="1" spans="1:17">
       <c r="A10" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>221</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>222</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>179</v>
@@ -4975,13 +4985,13 @@
         <v>56</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M10" s="3" t="s">
         <v>45</v>
@@ -5001,16 +5011,16 @@
     </row>
     <row r="11" ht="62" customHeight="1" spans="1:17">
       <c r="A11" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>226</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>227</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>179</v>
@@ -5025,16 +5035,16 @@
         <v>64</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M11" s="3" t="s">
         <v>45</v>
@@ -5054,16 +5064,16 @@
     </row>
     <row r="12" ht="62" customHeight="1" spans="1:17">
       <c r="A12" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>231</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>232</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>179</v>
@@ -5081,13 +5091,13 @@
         <v>41</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M12" s="3" t="s">
         <v>45</v>
@@ -5107,22 +5117,22 @@
     </row>
     <row r="13" ht="62" customHeight="1" spans="1:17">
       <c r="A13" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>237</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>179</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>49</v>
@@ -5134,22 +5144,20 @@
         <v>57</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="N13" s="3" t="s">
-        <v>45</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="N13" s="3"/>
       <c r="O13" s="3" t="s">
-        <v>45</v>
+        <v>131</v>
       </c>
       <c r="P13" s="3" t="s">
         <v>45</v>
@@ -5160,16 +5168,16 @@
     </row>
     <row r="14" ht="62" customHeight="1" spans="1:17">
       <c r="A14" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>241</v>
-      </c>
       <c r="C14" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>179</v>
@@ -5184,16 +5192,16 @@
         <v>64</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>45</v>
@@ -5213,16 +5221,16 @@
     </row>
     <row r="15" ht="62" customHeight="1" spans="1:17">
       <c r="A15" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>244</v>
-      </c>
       <c r="C15" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>179</v>
@@ -5240,13 +5248,13 @@
         <v>119</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L15" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M15" s="3" t="s">
         <v>45</v>
@@ -5266,16 +5274,16 @@
     </row>
     <row r="16" ht="62" customHeight="1" spans="1:17">
       <c r="A16" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>247</v>
-      </c>
       <c r="C16" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>179</v>
@@ -5293,13 +5301,13 @@
         <v>72</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>45</v>
@@ -5319,16 +5327,16 @@
     </row>
     <row r="17" ht="62" customHeight="1" spans="1:17">
       <c r="A17" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>250</v>
-      </c>
       <c r="C17" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>179</v>
@@ -5349,22 +5357,22 @@
         <v>45</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>184</v>
+        <v>44</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>45</v>
+        <v>141</v>
       </c>
       <c r="N17" s="3" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="P17" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="Q17" s="3" t="s">
         <v>45</v>
@@ -5372,16 +5380,16 @@
     </row>
     <row r="18" ht="62" customHeight="1" spans="1:17">
       <c r="A18" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>253</v>
-      </c>
       <c r="C18" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>179</v>
@@ -5399,13 +5407,13 @@
         <v>95</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>183</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M18" s="3" t="s">
         <v>45</v>
@@ -5458,7 +5466,7 @@
         <v>183</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>45</v>
@@ -5511,7 +5519,7 @@
         <v>183</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>45</v>
@@ -5564,7 +5572,7 @@
         <v>183</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M21" s="3" t="s">
         <v>45</v>
@@ -5617,7 +5625,7 @@
         <v>183</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>45</v>
@@ -5667,10 +5675,10 @@
         <v>45</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M23" s="3" t="s">
         <v>45</v>
@@ -5720,10 +5728,10 @@
         <v>45</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M24" s="3" t="s">
         <v>45</v>
@@ -5773,10 +5781,10 @@
         <v>45</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>45</v>
@@ -5829,7 +5837,7 @@
         <v>183</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>45</v>
@@ -5882,7 +5890,7 @@
         <v>183</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M27" s="3" t="s">
         <v>45</v>
@@ -5932,10 +5940,10 @@
         <v>45</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>45</v>
@@ -5988,7 +5996,7 @@
         <v>183</v>
       </c>
       <c r="L29" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M29" s="3" t="s">
         <v>45</v>
@@ -6038,10 +6046,10 @@
         <v>45</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L30" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M30" s="3" t="s">
         <v>45</v>
@@ -6091,10 +6099,10 @@
         <v>45</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M31" s="3" t="s">
         <v>45</v>
@@ -6144,10 +6152,10 @@
         <v>45</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L32" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M32" s="3" t="s">
         <v>45</v>
@@ -6197,10 +6205,10 @@
         <v>45</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M33" s="3" t="s">
         <v>45</v>
@@ -6250,10 +6258,10 @@
         <v>45</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L34" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M34" s="3" t="s">
         <v>45</v>
@@ -6303,10 +6311,10 @@
         <v>45</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L35" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M35" s="3" t="s">
         <v>45</v>
@@ -6356,10 +6364,10 @@
         <v>45</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L36" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M36" s="3" t="s">
         <v>45</v>
@@ -6409,10 +6417,10 @@
         <v>45</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L37" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M37" s="3" t="s">
         <v>45</v>
@@ -6462,10 +6470,10 @@
         <v>45</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L38" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M38" s="3" t="s">
         <v>45</v>
@@ -6515,10 +6523,10 @@
         <v>45</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L39" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M39" s="3" t="s">
         <v>45</v>
@@ -6568,10 +6576,10 @@
         <v>45</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L40" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M40" s="3" t="s">
         <v>45</v>
@@ -6621,10 +6629,10 @@
         <v>45</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M41" s="3" t="s">
         <v>45</v>
@@ -6674,10 +6682,10 @@
         <v>45</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L42" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M42" s="3" t="s">
         <v>45</v>
@@ -6727,10 +6735,10 @@
         <v>45</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M43" s="3" t="s">
         <v>45</v>
@@ -6780,10 +6788,10 @@
         <v>45</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L44" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M44" s="3" t="s">
         <v>45</v>
@@ -6836,7 +6844,7 @@
         <v>183</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>45</v>
@@ -6889,7 +6897,7 @@
         <v>183</v>
       </c>
       <c r="L46" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M46" s="3" t="s">
         <v>45</v>
@@ -6942,7 +6950,7 @@
         <v>183</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="M47" s="3" t="s">
         <v>45</v>
@@ -7009,9 +7017,9 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="2" max="2" width="26.4285714285714" customWidth="1"/>
     <col min="3" max="3" width="55" customWidth="1"/>
-    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="4" max="4" width="18.7142857142857" customWidth="1"/>
     <col min="5" max="5" width="55" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="55" customWidth="1"/>
@@ -7057,7 +7065,7 @@
         <v>349</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>45</v>
@@ -7080,7 +7088,7 @@
         <v>349</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>45</v>
@@ -7103,7 +7111,7 @@
         <v>349</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>45</v>
@@ -7126,7 +7134,7 @@
         <v>349</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>45</v>
@@ -7149,7 +7157,7 @@
         <v>349</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>45</v>
@@ -7172,7 +7180,7 @@
         <v>349</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>45</v>
@@ -7195,7 +7203,7 @@
         <v>349</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>45</v>
@@ -7218,7 +7226,7 @@
         <v>349</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>45</v>
@@ -7241,7 +7249,7 @@
         <v>349</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>45</v>
@@ -7264,7 +7272,7 @@
         <v>349</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>45</v>
@@ -7287,7 +7295,7 @@
         <v>349</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>45</v>
@@ -7310,7 +7318,7 @@
         <v>349</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>45</v>
@@ -7333,7 +7341,7 @@
         <v>349</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>45</v>
@@ -7356,7 +7364,7 @@
         <v>349</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>45</v>
@@ -7379,7 +7387,7 @@
         <v>349</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>45</v>
@@ -7402,7 +7410,7 @@
         <v>349</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>45</v>
@@ -7425,7 +7433,7 @@
         <v>349</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>45</v>
@@ -7448,7 +7456,7 @@
         <v>349</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G19" s="3" t="s">
         <v>45</v>
@@ -7471,7 +7479,7 @@
         <v>349</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G20" s="3" t="s">
         <v>45</v>
@@ -7494,7 +7502,7 @@
         <v>349</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G21" s="3" t="s">
         <v>45</v>
@@ -7517,7 +7525,7 @@
         <v>349</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G22" s="3" t="s">
         <v>45</v>
@@ -7540,7 +7548,7 @@
         <v>349</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G23" s="3" t="s">
         <v>45</v>
@@ -7563,7 +7571,7 @@
         <v>349</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G24" s="3" t="s">
         <v>45</v>
@@ -7586,7 +7594,7 @@
         <v>349</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G25" s="3" t="s">
         <v>45</v>
@@ -7609,7 +7617,7 @@
         <v>349</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G26" s="3" t="s">
         <v>45</v>
@@ -7632,7 +7640,7 @@
         <v>349</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G27" s="3" t="s">
         <v>45</v>
@@ -7655,7 +7663,7 @@
         <v>349</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G28" s="3" t="s">
         <v>45</v>
@@ -7678,7 +7686,7 @@
         <v>349</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G29" s="3" t="s">
         <v>45</v>
@@ -7701,7 +7709,7 @@
         <v>349</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G30" s="3" t="s">
         <v>45</v>
@@ -7724,7 +7732,7 @@
         <v>349</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G31" s="3" t="s">
         <v>45</v>
@@ -7747,7 +7755,7 @@
         <v>349</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G32" s="3" t="s">
         <v>45</v>
@@ -7770,7 +7778,7 @@
         <v>349</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G33" s="3" t="s">
         <v>45</v>
@@ -7793,7 +7801,7 @@
         <v>349</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G34" s="3" t="s">
         <v>45</v>
@@ -7816,7 +7824,7 @@
         <v>349</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G35" s="3" t="s">
         <v>45</v>
@@ -7839,7 +7847,7 @@
         <v>349</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G36" s="3" t="s">
         <v>45</v>
@@ -7862,7 +7870,7 @@
         <v>349</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G37" s="3" t="s">
         <v>45</v>
@@ -7885,7 +7893,7 @@
         <v>349</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G38" s="3" t="s">
         <v>45</v>
@@ -7908,7 +7916,7 @@
         <v>349</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G39" s="3" t="s">
         <v>45</v>
@@ -7931,7 +7939,7 @@
         <v>349</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G40" s="3" t="s">
         <v>45</v>
@@ -7954,7 +7962,7 @@
         <v>349</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G41" s="3" t="s">
         <v>45</v>
@@ -7977,7 +7985,7 @@
         <v>349</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G42" s="3" t="s">
         <v>45</v>
@@ -8000,7 +8008,7 @@
         <v>349</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G43" s="3" t="s">
         <v>45</v>
@@ -8023,7 +8031,7 @@
         <v>349</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G44" s="3" t="s">
         <v>45</v>
@@ -8046,7 +8054,7 @@
         <v>349</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G45" s="3" t="s">
         <v>45</v>
@@ -8069,7 +8077,7 @@
         <v>349</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G46" s="3" t="s">
         <v>45</v>
@@ -8092,7 +8100,7 @@
         <v>349</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G47" s="3" t="s">
         <v>45</v>
@@ -8115,7 +8123,7 @@
         <v>349</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G48" s="3" t="s">
         <v>45</v>
@@ -8138,7 +8146,7 @@
         <v>349</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G49" s="3" t="s">
         <v>45</v>
@@ -8161,7 +8169,7 @@
         <v>349</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G50" s="3" t="s">
         <v>45</v>
@@ -8184,7 +8192,7 @@
         <v>349</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G51" s="3" t="s">
         <v>45</v>
@@ -8207,7 +8215,7 @@
         <v>349</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G52" s="3" t="s">
         <v>45</v>
@@ -8230,7 +8238,7 @@
         <v>349</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G53" s="3" t="s">
         <v>45</v>
@@ -8253,7 +8261,7 @@
         <v>349</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G54" s="3" t="s">
         <v>45</v>
@@ -8276,7 +8284,7 @@
         <v>349</v>
       </c>
       <c r="F55" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G55" s="3" t="s">
         <v>45</v>
@@ -8299,7 +8307,7 @@
         <v>349</v>
       </c>
       <c r="F56" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G56" s="3" t="s">
         <v>45</v>
@@ -8322,7 +8330,7 @@
         <v>349</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>184</v>
+        <v>254</v>
       </c>
       <c r="G57" s="3" t="s">
         <v>45</v>
@@ -8348,9 +8356,9 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="2" width="19.4285714285714" customWidth="1"/>
+    <col min="3" max="3" width="14.8571428571429" customWidth="1"/>
     <col min="4" max="4" width="55" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="55" customWidth="1"/>

</xml_diff>